<commit_message>
Atualização da pasta do arquivo.
</commit_message>
<xml_diff>
--- a/excel_treino/src/main/resources/biblioteca.xlsx
+++ b/excel_treino/src/main/resources/biblioteca.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
   <si>
     <t>id</t>
   </si>
@@ -187,7 +187,7 @@
         <v>12</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">

</xml_diff>